<commit_message>
working on balance report
</commit_message>
<xml_diff>
--- a/application/plugins/StockSectorManager/views/stockBill.xlsx
+++ b/application/plugins/StockSectorManager/views/stockBill.xlsx
@@ -114,7 +114,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0;\-0;\-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -169,14 +169,6 @@
     <font>
       <b/>
       <sz val="16"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -311,7 +303,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>